<commit_message>
update May 2025 journey
</commit_message>
<xml_diff>
--- a/docs/journey/files/Travel History.xlsx
+++ b/docs/journey/files/Travel History.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lwyoh\myflightlog\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58BF3256-EDBE-4621-88CC-3683C63916DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A221B04-8FFC-481E-B843-917217487570}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="17496" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-19298" yWindow="-98" windowWidth="19396" windowHeight="12196" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="104">
   <si>
     <t>Country</t>
   </si>
@@ -325,6 +325,18 @@
   </si>
   <si>
     <t>St. Gallen</t>
+  </si>
+  <si>
+    <t>Ticino</t>
+  </si>
+  <si>
+    <t>2025-05</t>
+  </si>
+  <si>
+    <t>Nidwalden</t>
+  </si>
+  <si>
+    <t>Obwalden</t>
   </si>
 </sst>
 </file>
@@ -648,7 +660,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D50"/>
+  <dimension ref="A1:D53"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="11.109375" customWidth="1"/>
@@ -1355,6 +1367,48 @@
         <v>97</v>
       </c>
     </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>20</v>
+      </c>
+      <c r="B51" t="s">
+        <v>79</v>
+      </c>
+      <c r="C51" t="s">
+        <v>100</v>
+      </c>
+      <c r="D51" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>20</v>
+      </c>
+      <c r="B52" t="s">
+        <v>79</v>
+      </c>
+      <c r="C52" t="s">
+        <v>102</v>
+      </c>
+      <c r="D52" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>20</v>
+      </c>
+      <c r="B53" t="s">
+        <v>79</v>
+      </c>
+      <c r="C53" t="s">
+        <v>103</v>
+      </c>
+      <c r="D53" t="s">
+        <v>101</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>